<commit_message>
Liên kết số BBNT, ngày và đối tượng nghiệm thu của các phụ lục XD8 sang file danh mục
Các file 2-5 của mỗi đoạn tham chiếu sheet 'Tuyến XD8' trong file
'1. Danh mục nghiệm thu' cùng thư mục (external link, giống bộ HD5),
nên chỉ cần sửa ngày ở file danh mục.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RHahmApFFRr7mqf4R5YZ3w
</commit_message>
<xml_diff>
--- a/XD8/Đoạn 1/2. KL phân lớp cát đắp - XD8 đoạn 1.xlsx
+++ b/XD8/Đoạn 1/2. KL phân lớp cát đắp - XD8 đoạn 1.xlsx
@@ -18,6 +18,9 @@
     <sheet name="4.KTHH L4" sheetId="8" state="visible" r:id="rId10"/>
     <sheet name="4.KL lớp 4" sheetId="9" state="visible" r:id="rId11"/>
   </sheets>
+  <externalReferences>
+    <externalReference r:id="rIdExt1"/>
+  </externalReferences>
   <definedNames>
     <definedName function="false" hidden="false" localSheetId="2" name="_xlnm.Print_Area" vbProcedure="false">'1.KL lớp 1'!$A$1:$AB$60</definedName>
     <definedName function="false" hidden="false" localSheetId="1" name="_xlnm.Print_Area" vbProcedure="false">'1.KTHH L1'!$A$1:$S$71</definedName>
@@ -1104,6 +1107,432 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
+    <sheetNames>
+      <sheetName val="IN"/>
+      <sheetName val="Tuyến XD8"/>
+      <sheetName val="1. PL đường đen"/>
+      <sheetName val="2. Cao độ đào nền"/>
+      <sheetName val="2. KL đào nền"/>
+      <sheetName val="3. KTHH vải lọc"/>
+      <sheetName val="3. KL vải lọc"/>
+      <sheetName val="chạy VL"/>
+      <sheetName val="KL tưới nhựa"/>
+      <sheetName val="CĐ mặt đường"/>
+      <sheetName val="KL BTN"/>
+    </sheetNames>
+    <sheetDataSet>
+      <sheetData sheetId="0"/>
+      <sheetData sheetId="1">
+        <row r="3">
+          <cell r="A3">
+            <v>1</v>
+          </cell>
+          <cell r="B3" t="str">
+            <v xml:space="preserve">Kiểm tra cao độ đường đen đoạn từ Km0+224,25 -:- Km0+394,75</v>
+          </cell>
+          <cell r="D3" t="str">
+            <v xml:space="preserve">ngày 15 tháng 08 năm 2026</v>
+          </cell>
+          <cell r="G3" t="str">
+            <v xml:space="preserve">01.NĐXD8/CVXD </v>
+          </cell>
+        </row>
+        <row r="4">
+          <cell r="A4">
+            <v>2</v>
+          </cell>
+          <cell r="B4" t="str">
+            <v xml:space="preserve">Đào đất xử lý nền đường đoạn từ Km0+224,25 - Km0+394,75</v>
+          </cell>
+          <cell r="D4" t="str">
+            <v xml:space="preserve">ngày 16 tháng 08 năm 2026</v>
+          </cell>
+          <cell r="G4" t="str">
+            <v xml:space="preserve">02.NĐXD8/CVXD </v>
+          </cell>
+        </row>
+        <row r="5">
+          <cell r="A5">
+            <v>3</v>
+          </cell>
+          <cell r="B5" t="str">
+            <v xml:space="preserve">Rải vải địa kỹ thuật đoạn từ Km0+224,25 - Km0+394,75</v>
+          </cell>
+          <cell r="D5" t="str">
+            <v xml:space="preserve">ngày 17 tháng 08 năm 2026</v>
+          </cell>
+          <cell r="G5" t="str">
+            <v xml:space="preserve">03.NĐXD8/CVXD </v>
+          </cell>
+        </row>
+        <row r="6">
+          <cell r="A6">
+            <v>4</v>
+          </cell>
+          <cell r="B6" t="str">
+            <v xml:space="preserve">Đắp cát nền đường lớp 1 đoạn từ Km0+224,25 - Km0+394,75, độ chặt K&gt;=0,95</v>
+          </cell>
+          <cell r="D6" t="str">
+            <v xml:space="preserve">ngày 17 tháng 08 năm 2026</v>
+          </cell>
+          <cell r="G6" t="str">
+            <v xml:space="preserve">04.NĐXD8/CVXD </v>
+          </cell>
+        </row>
+        <row r="7">
+          <cell r="A7">
+            <v>5</v>
+          </cell>
+          <cell r="B7" t="str">
+            <v xml:space="preserve">Đắp cát nền đường lớp 2 đoạn từ Km0+224,25 - Km0+394,75, độ chặt K&gt;=0,95</v>
+          </cell>
+          <cell r="D7" t="str">
+            <v xml:space="preserve">ngày 18 tháng 08 năm 2026</v>
+          </cell>
+          <cell r="G7" t="str">
+            <v xml:space="preserve">05.NĐXD8/CVXD </v>
+          </cell>
+        </row>
+        <row r="8">
+          <cell r="A8">
+            <v>6</v>
+          </cell>
+          <cell r="B8" t="str">
+            <v xml:space="preserve">Đắp cát nền đường lớp 3 đoạn từ Km0+224,25 - Km0+394,75, độ chặt K&gt;=0,95</v>
+          </cell>
+          <cell r="D8" t="str">
+            <v xml:space="preserve">ngày 18 tháng 08 năm 2026</v>
+          </cell>
+          <cell r="G8" t="str">
+            <v xml:space="preserve">06.NĐXD8/CVXD </v>
+          </cell>
+        </row>
+        <row r="9">
+          <cell r="A9">
+            <v>7</v>
+          </cell>
+          <cell r="B9" t="str">
+            <v xml:space="preserve">Đắp cát nền đường lớp 4 đoạn từ Km0+224,25 - Km0+394,75, độ chặt K&gt;=0,95</v>
+          </cell>
+          <cell r="D9" t="str">
+            <v xml:space="preserve">ngày 19 tháng 08 năm 2026</v>
+          </cell>
+          <cell r="G9" t="str">
+            <v xml:space="preserve">07.NĐXD8/CVXD </v>
+          </cell>
+        </row>
+        <row r="10">
+          <cell r="A10">
+            <v>8</v>
+          </cell>
+          <cell r="B10" t="str">
+            <v xml:space="preserve">Đắp đất nền đường lớp 1 đoạn từ Km0+224,25 - Km0+394,75, độ chặt K&gt;=0,95</v>
+          </cell>
+          <cell r="D10" t="str">
+            <v xml:space="preserve">ngày 19 tháng 08 năm 2026</v>
+          </cell>
+          <cell r="G10" t="str">
+            <v xml:space="preserve">08.NĐXD8/CVXD </v>
+          </cell>
+        </row>
+        <row r="11">
+          <cell r="A11">
+            <v>9</v>
+          </cell>
+          <cell r="B11" t="str">
+            <v xml:space="preserve">Đắp đất nền đường lớp 2 đoạn từ Km0+224,25 - Km0+394,75, độ chặt K&gt;=0,95</v>
+          </cell>
+          <cell r="D11" t="str">
+            <v xml:space="preserve">ngày 20 tháng 08 năm 2026</v>
+          </cell>
+          <cell r="G11" t="str">
+            <v xml:space="preserve">09.NĐXD8/CVXD </v>
+          </cell>
+        </row>
+        <row r="12">
+          <cell r="A12">
+            <v>10</v>
+          </cell>
+          <cell r="B12" t="str">
+            <v xml:space="preserve">Đắp đất nền đường lớp 3 đoạn từ Km0+224,25 - Km0+394,75, độ chặt K&gt;=0,95</v>
+          </cell>
+          <cell r="D12" t="str">
+            <v xml:space="preserve">ngày 20 tháng 08 năm 2026</v>
+          </cell>
+          <cell r="G12" t="str">
+            <v xml:space="preserve">10.NĐXD8/CVXD </v>
+          </cell>
+        </row>
+        <row r="13">
+          <cell r="A13">
+            <v>11</v>
+          </cell>
+          <cell r="B13" t="str">
+            <v xml:space="preserve">Đắp đất nền đường lớp 4 đoạn từ Km0+224,25 - Km0+394,75, độ chặt K&gt;=0,95</v>
+          </cell>
+          <cell r="D13" t="str">
+            <v xml:space="preserve">ngày 21 tháng 08 năm 2026</v>
+          </cell>
+          <cell r="G13" t="str">
+            <v xml:space="preserve">11.NĐXD8/CVXD </v>
+          </cell>
+        </row>
+        <row r="14">
+          <cell r="A14">
+            <v>12</v>
+          </cell>
+          <cell r="B14" t="str">
+            <v xml:space="preserve">Đắp đất nền đường lớp 5 đoạn từ Km0+224,25 - Km0+394,75, độ chặt K&gt;=0,95</v>
+          </cell>
+          <cell r="D14" t="str">
+            <v xml:space="preserve">ngày 21 tháng 08 năm 2026</v>
+          </cell>
+          <cell r="G14" t="str">
+            <v xml:space="preserve">12.NĐXD8/CVXD </v>
+          </cell>
+        </row>
+        <row r="15">
+          <cell r="A15">
+            <v>13</v>
+          </cell>
+          <cell r="B15" t="str">
+            <v xml:space="preserve">Đắp đất nền đường lớp 6 đoạn từ Km0+224,25 - Km0+394,75, độ chặt K&gt;=0,95</v>
+          </cell>
+          <cell r="D15" t="str">
+            <v xml:space="preserve">ngày 22 tháng 08 năm 2026</v>
+          </cell>
+          <cell r="G15" t="str">
+            <v xml:space="preserve">13.NĐXD8/CVXD </v>
+          </cell>
+        </row>
+        <row r="16">
+          <cell r="A16">
+            <v>14</v>
+          </cell>
+          <cell r="B16" t="str">
+            <v xml:space="preserve">Đắp đất nền đường lớp 7 đoạn từ Km0+224,25 - Km0+394,75, độ chặt K&gt;=0,95</v>
+          </cell>
+          <cell r="D16" t="str">
+            <v xml:space="preserve">ngày 22 tháng 08 năm 2026</v>
+          </cell>
+          <cell r="G16" t="str">
+            <v xml:space="preserve">14.NĐXD8/CVXD </v>
+          </cell>
+        </row>
+        <row r="17">
+          <cell r="A17">
+            <v>15</v>
+          </cell>
+          <cell r="B17" t="str">
+            <v xml:space="preserve">Đắp đất nền đường lớp 8 đoạn từ Km0+224,25 - Km0+394,75, độ chặt K&gt;=0,95</v>
+          </cell>
+          <cell r="D17" t="str">
+            <v xml:space="preserve">ngày 23 tháng 08 năm 2026</v>
+          </cell>
+          <cell r="G17" t="str">
+            <v xml:space="preserve">15.NĐXD8/CVXD </v>
+          </cell>
+        </row>
+        <row r="18">
+          <cell r="A18">
+            <v>16</v>
+          </cell>
+          <cell r="B18" t="str">
+            <v xml:space="preserve">Đắp đất nền đường lớp 9 đoạn từ Km0+224,25 - Km0+394,75, độ chặt K&gt;=0,95</v>
+          </cell>
+          <cell r="D18" t="str">
+            <v xml:space="preserve">ngày 23 tháng 08 năm 2026</v>
+          </cell>
+          <cell r="G18" t="str">
+            <v xml:space="preserve">16.NĐXD8/CVXD </v>
+          </cell>
+        </row>
+        <row r="19">
+          <cell r="A19">
+            <v>17</v>
+          </cell>
+          <cell r="B19" t="str">
+            <v xml:space="preserve">Đắp đất nền đường lớp 1, độ chặt K&gt;=0,98 đoạn từ Km0+224,25 - Km0+394,75</v>
+          </cell>
+          <cell r="D19" t="str">
+            <v xml:space="preserve">ngày 24 tháng 08 năm 2026</v>
+          </cell>
+          <cell r="G19" t="str">
+            <v xml:space="preserve">17.NĐXD8/CVXD </v>
+          </cell>
+        </row>
+        <row r="20">
+          <cell r="A20">
+            <v>18</v>
+          </cell>
+          <cell r="B20" t="str">
+            <v xml:space="preserve">Đắp đất lề đường lớp 1, độ chặt K&gt;=0,95 đoạn từ Km0+224,25 - Km0+394,75</v>
+          </cell>
+          <cell r="D20" t="str">
+            <v xml:space="preserve">ngày 24 tháng 08 năm 2026</v>
+          </cell>
+          <cell r="G20" t="str">
+            <v xml:space="preserve">18.NĐXD8/CVXD </v>
+          </cell>
+        </row>
+        <row r="21">
+          <cell r="A21">
+            <v>19</v>
+          </cell>
+          <cell r="B21" t="str">
+            <v xml:space="preserve">Đắp đất nền đường lớp 2, độ chặt K&gt;=0,98 đoạn từ Km0+224,25 - Km0+394,75</v>
+          </cell>
+          <cell r="D21" t="str">
+            <v xml:space="preserve">ngày 25 tháng 08 năm 2026</v>
+          </cell>
+          <cell r="G21" t="str">
+            <v xml:space="preserve">19.NĐXD8/CVXD </v>
+          </cell>
+        </row>
+        <row r="22">
+          <cell r="A22">
+            <v>20</v>
+          </cell>
+          <cell r="B22" t="str">
+            <v xml:space="preserve">Đắp đất lề đường lớp 2, độ chặt K&gt;=0,95 đoạn từ Km0+224,25 - Km0+394,75</v>
+          </cell>
+          <cell r="D22" t="str">
+            <v xml:space="preserve">ngày 25 tháng 08 năm 2026</v>
+          </cell>
+          <cell r="G22" t="str">
+            <v xml:space="preserve">20.NĐXD8/CVXD </v>
+          </cell>
+        </row>
+        <row r="23">
+          <cell r="A23">
+            <v>21</v>
+          </cell>
+          <cell r="B23" t="str">
+            <v xml:space="preserve">Đắp cấp phối đá dăm loại 2 đoạn từ Km0+224,25 - Km0+394,75</v>
+          </cell>
+          <cell r="D23" t="str">
+            <v xml:space="preserve">ngày 26 tháng 08 năm 2026</v>
+          </cell>
+          <cell r="G23" t="str">
+            <v xml:space="preserve">21.NĐXD8/CVXD </v>
+          </cell>
+        </row>
+        <row r="24">
+          <cell r="A24">
+            <v>22</v>
+          </cell>
+          <cell r="B24" t="str">
+            <v xml:space="preserve">Đắp đất lề đường lớp 3, độ chặt K&gt;=0,95 đoạn từ Km0+224,25 - Km0+394,75</v>
+          </cell>
+          <cell r="D24" t="str">
+            <v xml:space="preserve">ngày 26 tháng 08 năm 2026</v>
+          </cell>
+          <cell r="G24" t="str">
+            <v xml:space="preserve">22.NĐXD8/CVXD </v>
+          </cell>
+        </row>
+        <row r="25">
+          <cell r="A25">
+            <v>23</v>
+          </cell>
+          <cell r="B25" t="str">
+            <v xml:space="preserve">Đắp đất lề đường lớp 4, độ chặt K&gt;=0,95 đoạn từ Km0+224,25 - Km0+394,75</v>
+          </cell>
+          <cell r="D25" t="str">
+            <v xml:space="preserve">ngày 27 tháng 08 năm 2026</v>
+          </cell>
+          <cell r="G25" t="str">
+            <v xml:space="preserve">23.NĐXD8/CVXD </v>
+          </cell>
+        </row>
+        <row r="26">
+          <cell r="A26">
+            <v>24</v>
+          </cell>
+          <cell r="B26" t="str">
+            <v xml:space="preserve">Đắp cấp phối đá dăm loại 1 đoạn từ Km0+224,25 - Km0+394,75</v>
+          </cell>
+          <cell r="D26" t="str">
+            <v xml:space="preserve">ngày 27 tháng 08 năm 2026</v>
+          </cell>
+          <cell r="G26" t="str">
+            <v xml:space="preserve">24.NĐXD8/CVXD </v>
+          </cell>
+        </row>
+        <row r="27">
+          <cell r="A27">
+            <v>25</v>
+          </cell>
+          <cell r="B27" t="str">
+            <v xml:space="preserve">Vệ sinh, thổi bụi mặt đường </v>
+          </cell>
+          <cell r="D27" t="str">
+            <v xml:space="preserve">ngày 29 tháng 08 năm 2026</v>
+          </cell>
+          <cell r="G27" t="str">
+            <v xml:space="preserve">25.NĐXD8/CVXD </v>
+          </cell>
+        </row>
+        <row r="28">
+          <cell r="A28">
+            <v>26</v>
+          </cell>
+          <cell r="B28" t="str">
+            <v xml:space="preserve">Tưới lớp thấm bám mặt đường, nhựa MC70, lượng nhựa 1kg/m2</v>
+          </cell>
+          <cell r="D28" t="str">
+            <v xml:space="preserve">ngày 31 tháng 08 năm 2026</v>
+          </cell>
+          <cell r="G28" t="str">
+            <v xml:space="preserve">26.NĐXD8/CVXD </v>
+          </cell>
+        </row>
+        <row r="29">
+          <cell r="A29">
+            <v>27</v>
+          </cell>
+          <cell r="B29" t="str">
+            <v xml:space="preserve">Rải thảm mặt đường bê tông nhựa C16 - Chiều dày mặt đường đã lèn ép 6cm</v>
+          </cell>
+          <cell r="D29" t="str">
+            <v xml:space="preserve">ngày 03 tháng 09 năm 2026</v>
+          </cell>
+          <cell r="G29" t="str">
+            <v xml:space="preserve">27.NĐXD8/CVXD </v>
+          </cell>
+        </row>
+        <row r="30">
+          <cell r="A30">
+            <v>28</v>
+          </cell>
+          <cell r="B30" t="str">
+            <v xml:space="preserve">Bê tông nhựa C16 - Chiều dày mặt đường đã lèn ép 6cm</v>
+          </cell>
+          <cell r="D30" t="str">
+            <v xml:space="preserve">ngày 05 tháng 09 năm 2026</v>
+          </cell>
+          <cell r="G30" t="str">
+            <v xml:space="preserve">28.NĐXD8/CVXD </v>
+          </cell>
+        </row>
+      </sheetData>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4"/>
+      <sheetData sheetId="5"/>
+      <sheetData sheetId="6"/>
+      <sheetData sheetId="7"/>
+      <sheetData sheetId="8"/>
+      <sheetData sheetId="9"/>
+      <sheetData sheetId="10"/>
+    </sheetDataSet>
+  </externalBook>
+</externalLink>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
   <a:themeElements>
@@ -3241,8 +3670,9 @@
       <c r="W1" s="4"/>
     </row>
     <row r="2" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5" t="s">
-        <v>29</v>
+      <c r="A2" s="5" t="str">
+        <f>"Kèm theo BBNT số: "&amp;VLOOKUP(AZ2,'[1]Tuyến XD8'!$A$2:$G$60,7,0)&amp;VLOOKUP(AZ2,'[1]Tuyến XD8'!$A$2:$G$60,4,0)</f>
+        <v xml:space="preserve">Kèm theo BBNT số: 04.NĐXD8/CVXD ngày 17 tháng 08 năm 2026</v>
       </c>
       <c r="B2" s="5"/>
       <c r="C2" s="5"/>
@@ -3266,6 +3696,9 @@
       <c r="U2" s="7"/>
       <c r="V2" s="7"/>
       <c r="W2" s="7"/>
+      <c r="AZ2">
+        <v>4</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
@@ -3379,8 +3812,9 @@
       <c r="D7" s="8"/>
       <c r="E7" s="8"/>
       <c r="F7" s="8"/>
-      <c r="G7" s="8" t="s">
-        <v>35</v>
+      <c r="G7" s="8" t="str">
+        <f>VLOOKUP(AZ2,'[1]Tuyến XD8'!$A$2:$B$60,2,0)</f>
+        <v xml:space="preserve">Đắp cát nền đường lớp 1 đoạn từ Km0+224,25 - Km0+394,75, độ chặt K&gt;=0,95</v>
       </c>
       <c r="H7" s="8"/>
       <c r="I7" s="8"/>
@@ -5175,8 +5609,9 @@
       <c r="AE1" s="3"/>
     </row>
     <row r="2" s="26" customFormat="true" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="27" t="s">
-        <v>29</v>
+      <c r="A2" s="27" t="str">
+        <f>"Kèm theo BBNT số: "&amp;VLOOKUP(AZ2,'[1]Tuyến XD8'!$A$2:$G$60,7,0)&amp;VLOOKUP(AZ2,'[1]Tuyến XD8'!$A$2:$G$60,4,0)</f>
+        <v xml:space="preserve">Kèm theo BBNT số: 04.NĐXD8/CVXD ngày 17 tháng 08 năm 2026</v>
       </c>
       <c r="B2" s="27"/>
       <c r="C2" s="27"/>
@@ -5207,6 +5642,9 @@
       <c r="AB2" s="27"/>
       <c r="AD2" s="6"/>
       <c r="AE2" s="7"/>
+      <c r="AZ2">
+        <v>4</v>
+      </c>
     </row>
     <row r="3" s="30" customFormat="true" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="28" t="s">
@@ -6153,8 +6591,9 @@
         <v>34</v>
       </c>
       <c r="B7" s="32"/>
-      <c r="D7" s="33" t="s">
-        <v>35</v>
+      <c r="D7" s="33" t="str">
+        <f>VLOOKUP(AZ2,'[1]Tuyến XD8'!$A$2:$B$60,2,0)</f>
+        <v xml:space="preserve">Đắp cát nền đường lớp 1 đoạn từ Km0+224,25 - Km0+394,75, độ chặt K&gt;=0,95</v>
       </c>
       <c r="E7" s="33"/>
       <c r="F7" s="33"/>
@@ -10823,8 +11262,9 @@
       <c r="W1" s="4"/>
     </row>
     <row r="2" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5" t="s">
-        <v>63</v>
+      <c r="A2" s="5" t="str">
+        <f>"Kèm theo BBNT số: "&amp;VLOOKUP(AZ2,'[1]Tuyến XD8'!$A$2:$G$60,7,0)&amp;VLOOKUP(AZ2,'[1]Tuyến XD8'!$A$2:$G$60,4,0)</f>
+        <v xml:space="preserve">Kèm theo BBNT số: 05.NĐXD8/CVXD ngày 18 tháng 08 năm 2026</v>
       </c>
       <c r="B2" s="5"/>
       <c r="C2" s="5"/>
@@ -10848,6 +11288,9 @@
       <c r="U2" s="7"/>
       <c r="V2" s="7"/>
       <c r="W2" s="7"/>
+      <c r="AZ2">
+        <v>5</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
@@ -10961,8 +11404,9 @@
       <c r="D7" s="8"/>
       <c r="E7" s="8"/>
       <c r="F7" s="8"/>
-      <c r="G7" s="8" t="s">
-        <v>64</v>
+      <c r="G7" s="8" t="str">
+        <f>VLOOKUP(AZ2,'[1]Tuyến XD8'!$A$2:$B$60,2,0)</f>
+        <v xml:space="preserve">Đắp cát nền đường lớp 2 đoạn từ Km0+224,25 - Km0+394,75, độ chặt K&gt;=0,95</v>
       </c>
       <c r="H7" s="8"/>
       <c r="I7" s="8"/>
@@ -12724,8 +13168,9 @@
       <c r="AE1" s="3"/>
     </row>
     <row r="2" s="26" customFormat="true" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="27" t="s">
-        <v>63</v>
+      <c r="A2" s="27" t="str">
+        <f>"Kèm theo BBNT số: "&amp;VLOOKUP(AZ2,'[1]Tuyến XD8'!$A$2:$G$60,7,0)&amp;VLOOKUP(AZ2,'[1]Tuyến XD8'!$A$2:$G$60,4,0)</f>
+        <v xml:space="preserve">Kèm theo BBNT số: 05.NĐXD8/CVXD ngày 18 tháng 08 năm 2026</v>
       </c>
       <c r="B2" s="27"/>
       <c r="C2" s="27"/>
@@ -12754,6 +13199,9 @@
       <c r="Z2" s="27"/>
       <c r="AA2" s="27"/>
       <c r="AB2" s="27"/>
+      <c r="AZ2">
+        <v>5</v>
+      </c>
     </row>
     <row r="3" s="30" customFormat="true" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="28" t="s">
@@ -13700,8 +14148,9 @@
         <v>34</v>
       </c>
       <c r="B7" s="32"/>
-      <c r="D7" s="33" t="s">
-        <v>64</v>
+      <c r="D7" s="33" t="str">
+        <f>VLOOKUP(AZ2,'[1]Tuyến XD8'!$A$2:$B$60,2,0)</f>
+        <v xml:space="preserve">Đắp cát nền đường lớp 2 đoạn từ Km0+224,25 - Km0+394,75, độ chặt K&gt;=0,95</v>
       </c>
       <c r="E7" s="33"/>
       <c r="F7" s="33"/>
@@ -18368,8 +18817,9 @@
       <c r="W1" s="4"/>
     </row>
     <row r="2" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5" t="s">
-        <v>65</v>
+      <c r="A2" s="5" t="str">
+        <f>"Kèm theo BBNT số: "&amp;VLOOKUP(AZ2,'[1]Tuyến XD8'!$A$2:$G$60,7,0)&amp;VLOOKUP(AZ2,'[1]Tuyến XD8'!$A$2:$G$60,4,0)</f>
+        <v xml:space="preserve">Kèm theo BBNT số: 06.NĐXD8/CVXD ngày 18 tháng 08 năm 2026</v>
       </c>
       <c r="B2" s="5"/>
       <c r="C2" s="5"/>
@@ -18392,6 +18842,9 @@
       <c r="U2" s="7"/>
       <c r="V2" s="7"/>
       <c r="W2" s="7"/>
+      <c r="AZ2">
+        <v>6</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
@@ -18505,8 +18958,9 @@
       <c r="D7" s="8"/>
       <c r="E7" s="8"/>
       <c r="F7" s="8"/>
-      <c r="G7" s="8" t="s">
-        <v>66</v>
+      <c r="G7" s="8" t="str">
+        <f>VLOOKUP(AZ2,'[1]Tuyến XD8'!$A$2:$B$60,2,0)</f>
+        <v xml:space="preserve">Đắp cát nền đường lớp 3 đoạn từ Km0+224,25 - Km0+394,75, độ chặt K&gt;=0,95</v>
       </c>
       <c r="H7" s="8"/>
       <c r="I7" s="8"/>
@@ -19953,8 +20407,9 @@
       <c r="AE1" s="3"/>
     </row>
     <row r="2" s="26" customFormat="true" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="27" t="s">
-        <v>65</v>
+      <c r="A2" s="27" t="str">
+        <f>"Kèm theo BBNT số: "&amp;VLOOKUP(AZ2,'[1]Tuyến XD8'!$A$2:$G$60,7,0)&amp;VLOOKUP(AZ2,'[1]Tuyến XD8'!$A$2:$G$60,4,0)</f>
+        <v xml:space="preserve">Kèm theo BBNT số: 06.NĐXD8/CVXD ngày 18 tháng 08 năm 2026</v>
       </c>
       <c r="B2" s="27"/>
       <c r="C2" s="27"/>
@@ -19984,6 +20439,9 @@
       <c r="AA2" s="27"/>
       <c r="AB2" s="27"/>
       <c r="AE2" s="7"/>
+      <c r="AZ2">
+        <v>6</v>
+      </c>
     </row>
     <row r="3" s="30" customFormat="true" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="28" t="s">
@@ -20930,8 +21388,9 @@
         <v>34</v>
       </c>
       <c r="B7" s="32"/>
-      <c r="D7" s="33" t="s">
-        <v>66</v>
+      <c r="D7" s="33" t="str">
+        <f>VLOOKUP(AZ2,'[1]Tuyến XD8'!$A$2:$B$60,2,0)</f>
+        <v xml:space="preserve">Đắp cát nền đường lớp 3 đoạn từ Km0+224,25 - Km0+394,75, độ chặt K&gt;=0,95</v>
       </c>
       <c r="E7" s="33"/>
       <c r="F7" s="33"/>
@@ -25118,8 +25577,9 @@
       <c r="W1" s="4"/>
     </row>
     <row r="2" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5" t="s">
-        <v>67</v>
+      <c r="A2" s="5" t="str">
+        <f>"Kèm theo BBNT số: "&amp;VLOOKUP(AZ2,'[1]Tuyến XD8'!$A$2:$G$60,7,0)&amp;VLOOKUP(AZ2,'[1]Tuyến XD8'!$A$2:$G$60,4,0)</f>
+        <v xml:space="preserve">Kèm theo BBNT số: 07.NĐXD8/CVXD ngày 19 tháng 08 năm 2026</v>
       </c>
       <c r="B2" s="5"/>
       <c r="C2" s="5"/>
@@ -25143,6 +25603,9 @@
       <c r="U2" s="74"/>
       <c r="V2" s="7"/>
       <c r="W2" s="7"/>
+      <c r="AZ2">
+        <v>7</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="8" t="s">
@@ -25256,8 +25719,9 @@
       <c r="D7" s="8"/>
       <c r="E7" s="8"/>
       <c r="F7" s="8"/>
-      <c r="G7" s="8" t="s">
-        <v>68</v>
+      <c r="G7" s="8" t="str">
+        <f>VLOOKUP(AZ2,'[1]Tuyến XD8'!$A$2:$B$60,2,0)</f>
+        <v xml:space="preserve">Đắp cát nền đường lớp 4 đoạn từ Km0+224,25 - Km0+394,75, độ chặt K&gt;=0,95</v>
       </c>
       <c r="H7" s="8"/>
       <c r="I7" s="8"/>
@@ -26726,8 +27190,9 @@
       <c r="AE1" s="3"/>
     </row>
     <row r="2" s="26" customFormat="true" ht="16.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="27" t="s">
-        <v>67</v>
+      <c r="A2" s="27" t="str">
+        <f>"Kèm theo BBNT số: "&amp;VLOOKUP(AZ2,'[1]Tuyến XD8'!$A$2:$G$60,7,0)&amp;VLOOKUP(AZ2,'[1]Tuyến XD8'!$A$2:$G$60,4,0)</f>
+        <v xml:space="preserve">Kèm theo BBNT số: 07.NĐXD8/CVXD ngày 19 tháng 08 năm 2026</v>
       </c>
       <c r="B2" s="27"/>
       <c r="C2" s="27"/>
@@ -26756,6 +27221,9 @@
       <c r="Z2" s="27"/>
       <c r="AA2" s="27"/>
       <c r="AB2" s="27"/>
+      <c r="AZ2">
+        <v>7</v>
+      </c>
     </row>
     <row r="3" s="30" customFormat="true" ht="37.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="28" t="s">
@@ -27702,8 +28170,9 @@
         <v>34</v>
       </c>
       <c r="B7" s="32"/>
-      <c r="D7" s="33" t="s">
-        <v>68</v>
+      <c r="D7" s="33" t="str">
+        <f>VLOOKUP(AZ2,'[1]Tuyến XD8'!$A$2:$B$60,2,0)</f>
+        <v xml:space="preserve">Đắp cát nền đường lớp 4 đoạn từ Km0+224,25 - Km0+394,75, độ chặt K&gt;=0,95</v>
       </c>
       <c r="E7" s="33"/>
       <c r="F7" s="33"/>

</xml_diff>